<commit_message>
Tabulasi Rp/km per rute: tambah asal (Jakarta) di semua lembar
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hasil_scraping/261009-Rp per km per Rute.xlsx
+++ b/hasil_scraping/261009-Rp per km per Rute.xlsx
@@ -117,8 +117,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -497,20 +497,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,6 +528,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Asal: Jakarta (CGK dan HLP); jarak dihitung dari CGK. Semua rute sekali jalan Jakarta → tujuan.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -535,50 +543,55 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Rute</t>
+          <t>Asal</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Kota</t>
+          <t>Tujuan</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>Kota tujuan</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>Jenis</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Jarak (km)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Jumlah penerbangan</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Harga rata-rata (Rp)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Rp/km rata-rata</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Rp/km median</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Rp/km minimum</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Rp/km maksimum</t>
         </is>
@@ -590,38 +603,43 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
           <t>KNO</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Medan</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Domestik</t>
         </is>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="F5" s="7" t="n">
         <v>1387</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="G5" s="7" t="n">
         <v>6973</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="H5" s="7" t="n">
         <v>2236209</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="I5" s="8" t="n">
         <v>1612</v>
       </c>
-      <c r="I5" s="7" t="n">
+      <c r="J5" s="7" t="n">
         <v>1597</v>
       </c>
-      <c r="J5" s="7" t="n">
+      <c r="K5" s="7" t="n">
         <v>933</v>
       </c>
-      <c r="K5" s="7" t="n">
+      <c r="L5" s="7" t="n">
         <v>2444</v>
       </c>
     </row>
@@ -631,38 +649,43 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
           <t>UPG</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Makassar</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Domestik</t>
         </is>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="F6" s="7" t="n">
         <v>1432</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="G6" s="7" t="n">
         <v>5722</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="H6" s="7" t="n">
         <v>2379080</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="I6" s="8" t="n">
         <v>1661</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="J6" s="7" t="n">
         <v>1659</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="K6" s="7" t="n">
         <v>803</v>
       </c>
-      <c r="K6" s="7" t="n">
+      <c r="L6" s="7" t="n">
         <v>4558</v>
       </c>
     </row>
@@ -672,38 +695,43 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
           <t>BPN</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Balikpapan</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Domestik</t>
         </is>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="F7" s="7" t="n">
         <v>1258</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="G7" s="7" t="n">
         <v>3053</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="H7" s="7" t="n">
         <v>2153555</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="I7" s="8" t="n">
         <v>1712</v>
       </c>
-      <c r="I7" s="7" t="n">
+      <c r="J7" s="7" t="n">
         <v>1671</v>
       </c>
-      <c r="J7" s="7" t="n">
+      <c r="K7" s="7" t="n">
         <v>1008</v>
       </c>
-      <c r="K7" s="7" t="n">
+      <c r="L7" s="7" t="n">
         <v>2273</v>
       </c>
     </row>
@@ -713,38 +741,43 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
           <t>PKU</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Pekanbaru</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Domestik</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="F8" s="7" t="n">
         <v>933</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="G8" s="7" t="n">
         <v>3809</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="H8" s="7" t="n">
         <v>1848350</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="I8" s="8" t="n">
         <v>1981</v>
       </c>
-      <c r="I8" s="7" t="n">
+      <c r="J8" s="7" t="n">
         <v>1928</v>
       </c>
-      <c r="J8" s="7" t="n">
+      <c r="K8" s="7" t="n">
         <v>1120</v>
       </c>
-      <c r="K8" s="7" t="n">
+      <c r="L8" s="7" t="n">
         <v>2721</v>
       </c>
     </row>
@@ -754,38 +787,43 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
           <t>DPS</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Denpasar</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Domestik</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="F9" s="7" t="n">
         <v>983</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="G9" s="7" t="n">
         <v>8686</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="H9" s="7" t="n">
         <v>2056056</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="I9" s="8" t="n">
         <v>2092</v>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="J9" s="7" t="n">
         <v>2030</v>
       </c>
-      <c r="J9" s="7" t="n">
+      <c r="K9" s="7" t="n">
         <v>995</v>
       </c>
-      <c r="K9" s="7" t="n">
+      <c r="L9" s="7" t="n">
         <v>3015</v>
       </c>
     </row>
@@ -795,38 +833,43 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
           <t>SUB</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Surabaya</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Domestik</t>
         </is>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="F10" s="7" t="n">
         <v>691</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="G10" s="7" t="n">
         <v>7974</v>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="H10" s="7" t="n">
         <v>1689246</v>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="I10" s="8" t="n">
         <v>2445</v>
       </c>
-      <c r="I10" s="7" t="n">
+      <c r="J10" s="7" t="n">
         <v>2458</v>
       </c>
-      <c r="J10" s="7" t="n">
+      <c r="K10" s="7" t="n">
         <v>1269</v>
       </c>
-      <c r="K10" s="7" t="n">
+      <c r="L10" s="7" t="n">
         <v>3383</v>
       </c>
     </row>
@@ -836,38 +879,43 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
           <t>YIA</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Yogyakarta</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Domestik</t>
         </is>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="F11" s="7" t="n">
         <v>424</v>
       </c>
-      <c r="F11" s="7" t="n">
+      <c r="G11" s="7" t="n">
         <v>3295</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="H11" s="7" t="n">
         <v>1339079</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="I11" s="8" t="n">
         <v>3158</v>
       </c>
-      <c r="I11" s="7" t="n">
+      <c r="J11" s="7" t="n">
         <v>3079</v>
       </c>
-      <c r="J11" s="7" t="n">
+      <c r="K11" s="7" t="n">
         <v>1439</v>
       </c>
-      <c r="K11" s="7" t="n">
+      <c r="L11" s="7" t="n">
         <v>4261</v>
       </c>
     </row>
@@ -877,38 +925,43 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
           <t>KUL</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Kuala Lumpur</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="F13" s="7" t="n">
         <v>1129</v>
       </c>
-      <c r="F13" s="7" t="n">
+      <c r="G13" s="7" t="n">
         <v>7443</v>
       </c>
-      <c r="G13" s="7" t="n">
+      <c r="H13" s="7" t="n">
         <v>2209956</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="I13" s="8" t="n">
         <v>1957</v>
       </c>
-      <c r="I13" s="7" t="n">
+      <c r="J13" s="7" t="n">
         <v>1781</v>
       </c>
-      <c r="J13" s="7" t="n">
+      <c r="K13" s="7" t="n">
         <v>641</v>
       </c>
-      <c r="K13" s="7" t="n">
+      <c r="L13" s="7" t="n">
         <v>9751</v>
       </c>
     </row>
@@ -918,38 +971,43 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
           <t>SIN</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Singapura</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="F14" s="7" t="n">
         <v>884</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="G14" s="7" t="n">
         <v>7199</v>
       </c>
-      <c r="G14" s="7" t="n">
+      <c r="H14" s="7" t="n">
         <v>2604305</v>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="I14" s="8" t="n">
         <v>2946</v>
       </c>
-      <c r="I14" s="7" t="n">
+      <c r="J14" s="7" t="n">
         <v>2445</v>
       </c>
-      <c r="J14" s="7" t="n">
+      <c r="K14" s="7" t="n">
         <v>692</v>
       </c>
-      <c r="K14" s="7" t="n">
+      <c r="L14" s="7" t="n">
         <v>16747</v>
       </c>
     </row>
@@ -1000,6 +1058,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Asal: Jakarta (CGK dan HLP); jarak dihitung dari CGK. Semua rute sekali jalan Jakarta → tujuan.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1008,44 +1073,44 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>BPN
-Balikpapan</t>
+          <t>Jakarta →
+BPN Balikpapan</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>DPS
-Denpasar</t>
+          <t>Jakarta →
+DPS Denpasar</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>KNO
-Medan</t>
+          <t>Jakarta →
+KNO Medan</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>PKU
-Pekanbaru</t>
+          <t>Jakarta →
+PKU Pekanbaru</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>SUB
-Surabaya</t>
+          <t>Jakarta →
+SUB Surabaya</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>UPG
-Makassar</t>
+          <t>Jakarta →
+UPG Makassar</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>YIA
-Yogyakarta</t>
+          <t>Jakarta →
+YIA Yogyakarta</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -1060,7 +1125,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>2022-08</t>
         </is>
@@ -1093,14 +1158,14 @@
       <c r="I5" s="8" t="n">
         <v>1145</v>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>2022-09</t>
         </is>
@@ -1133,14 +1198,14 @@
       <c r="I6" s="8" t="n">
         <v>1117</v>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>2022-10</t>
         </is>
@@ -1173,14 +1238,14 @@
       <c r="I7" s="8" t="n">
         <v>1083</v>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>2022-11</t>
         </is>
@@ -1213,14 +1278,14 @@
       <c r="I8" s="8" t="n">
         <v>1043</v>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>2022-12</t>
         </is>
@@ -1253,14 +1318,14 @@
       <c r="I9" s="8" t="n">
         <v>1094</v>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>2023-01</t>
         </is>
@@ -1293,14 +1358,14 @@
       <c r="I10" s="8" t="n">
         <v>946</v>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>2023-02</t>
         </is>
@@ -1333,14 +1398,14 @@
       <c r="I11" s="8" t="n">
         <v>829</v>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>2023-03</t>
         </is>
@@ -1373,14 +1438,14 @@
       <c r="I12" s="8" t="n">
         <v>871</v>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>2023-04</t>
         </is>
@@ -1413,14 +1478,14 @@
       <c r="I13" s="8" t="n">
         <v>845</v>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>2023-05</t>
         </is>
@@ -1453,14 +1518,14 @@
       <c r="I14" s="8" t="n">
         <v>810</v>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>2023-06</t>
         </is>
@@ -1493,14 +1558,14 @@
       <c r="I15" s="8" t="n">
         <v>832</v>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>2023-07</t>
         </is>
@@ -1533,14 +1598,14 @@
       <c r="I16" s="8" t="n">
         <v>890</v>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>2023-08</t>
         </is>
@@ -1573,14 +1638,14 @@
       <c r="I17" s="8" t="n">
         <v>921</v>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>2023-09</t>
         </is>
@@ -1613,14 +1678,14 @@
       <c r="I18" s="8" t="n">
         <v>938</v>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>2023-10</t>
         </is>
@@ -1651,14 +1716,14 @@
       <c r="I19" s="8" t="n">
         <v>1319</v>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>2023-11</t>
         </is>
@@ -1687,14 +1752,14 @@
       <c r="I20" s="8" t="n">
         <v>1428</v>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>2023-12</t>
         </is>
@@ -1723,14 +1788,14 @@
       <c r="I21" s="8" t="n">
         <v>1567</v>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J21" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>2024-01</t>
         </is>
@@ -1759,14 +1824,14 @@
       <c r="I22" s="8" t="n">
         <v>1443</v>
       </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>2024-02</t>
         </is>
@@ -1795,14 +1860,14 @@
       <c r="I23" s="8" t="n">
         <v>1438</v>
       </c>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>2024-03</t>
         </is>
@@ -1831,14 +1896,14 @@
       <c r="I24" s="8" t="n">
         <v>1439</v>
       </c>
-      <c r="J24" s="6" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>2024-04</t>
         </is>
@@ -1867,14 +1932,14 @@
       <c r="I25" s="8" t="n">
         <v>1570</v>
       </c>
-      <c r="J25" s="6" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>2024-05</t>
         </is>
@@ -1903,14 +1968,14 @@
       <c r="I26" s="8" t="n">
         <v>1484</v>
       </c>
-      <c r="J26" s="6" t="inlineStr">
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>2024-06</t>
         </is>
@@ -1939,14 +2004,14 @@
       <c r="I27" s="8" t="n">
         <v>1597</v>
       </c>
-      <c r="J27" s="6" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>2024-07</t>
         </is>
@@ -1975,14 +2040,14 @@
       <c r="I28" s="8" t="n">
         <v>1563</v>
       </c>
-      <c r="J28" s="6" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>2024-08</t>
         </is>
@@ -2011,14 +2076,14 @@
       <c r="I29" s="8" t="n">
         <v>1601</v>
       </c>
-      <c r="J29" s="6" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>2024-09</t>
         </is>
@@ -2047,14 +2112,14 @@
       <c r="I30" s="8" t="n">
         <v>1707</v>
       </c>
-      <c r="J30" s="6" t="inlineStr">
+      <c r="J30" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>2024-10</t>
         </is>
@@ -2083,14 +2148,14 @@
       <c r="I31" s="8" t="n">
         <v>1620</v>
       </c>
-      <c r="J31" s="6" t="inlineStr">
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>2024-11</t>
         </is>
@@ -2119,14 +2184,14 @@
       <c r="I32" s="8" t="n">
         <v>1638</v>
       </c>
-      <c r="J32" s="6" t="inlineStr">
+      <c r="J32" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>2024-12</t>
         </is>
@@ -2155,14 +2220,14 @@
       <c r="I33" s="8" t="n">
         <v>1717</v>
       </c>
-      <c r="J33" s="6" t="inlineStr">
+      <c r="J33" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
@@ -2191,14 +2256,14 @@
       <c r="I34" s="8" t="n">
         <v>1685</v>
       </c>
-      <c r="J34" s="6" t="inlineStr">
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>2025-02</t>
         </is>
@@ -2227,14 +2292,14 @@
       <c r="I35" s="8" t="n">
         <v>1827</v>
       </c>
-      <c r="J35" s="6" t="inlineStr">
+      <c r="J35" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>2025-03</t>
         </is>
@@ -2263,14 +2328,14 @@
       <c r="I36" s="8" t="n">
         <v>1798</v>
       </c>
-      <c r="J36" s="6" t="inlineStr">
+      <c r="J36" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>2025-04</t>
         </is>
@@ -2299,14 +2364,14 @@
       <c r="I37" s="8" t="n">
         <v>1682</v>
       </c>
-      <c r="J37" s="6" t="inlineStr">
+      <c r="J37" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
@@ -2335,14 +2400,14 @@
       <c r="I38" s="8" t="n">
         <v>1260</v>
       </c>
-      <c r="J38" s="6" t="inlineStr">
+      <c r="J38" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>2025-06</t>
         </is>
@@ -2371,14 +2436,14 @@
       <c r="I39" s="8" t="n">
         <v>1412</v>
       </c>
-      <c r="J39" s="6" t="inlineStr">
+      <c r="J39" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>2025-07</t>
         </is>
@@ -2407,14 +2472,14 @@
       <c r="I40" s="8" t="n">
         <v>1392</v>
       </c>
-      <c r="J40" s="6" t="inlineStr">
+      <c r="J40" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>2025-08</t>
         </is>
@@ -2443,14 +2508,14 @@
       <c r="I41" s="8" t="n">
         <v>1353</v>
       </c>
-      <c r="J41" s="6" t="inlineStr">
+      <c r="J41" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
@@ -2479,14 +2544,14 @@
       <c r="I42" s="8" t="n">
         <v>1383</v>
       </c>
-      <c r="J42" s="6" t="inlineStr">
+      <c r="J42" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>2025-10</t>
         </is>
@@ -2515,14 +2580,14 @@
       <c r="I43" s="8" t="n">
         <v>1116</v>
       </c>
-      <c r="J43" s="6" t="inlineStr">
+      <c r="J43" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>2025-11</t>
         </is>
@@ -2551,14 +2616,14 @@
       <c r="I44" s="8" t="n">
         <v>1109</v>
       </c>
-      <c r="J44" s="6" t="inlineStr">
+      <c r="J44" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
@@ -2587,14 +2652,14 @@
       <c r="I45" s="8" t="n">
         <v>1304</v>
       </c>
-      <c r="J45" s="6" t="inlineStr">
+      <c r="J45" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
@@ -2623,14 +2688,14 @@
       <c r="I46" s="8" t="n">
         <v>1178</v>
       </c>
-      <c r="J46" s="6" t="inlineStr">
+      <c r="J46" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
@@ -2659,14 +2724,14 @@
       <c r="I47" s="8" t="n">
         <v>1254</v>
       </c>
-      <c r="J47" s="6" t="inlineStr">
+      <c r="J47" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
@@ -2695,14 +2760,14 @@
       <c r="I48" s="8" t="n">
         <v>1306</v>
       </c>
-      <c r="J48" s="6" t="inlineStr">
+      <c r="J48" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
@@ -2731,14 +2796,14 @@
       <c r="I49" s="8" t="n">
         <v>1346</v>
       </c>
-      <c r="J49" s="6" t="inlineStr">
+      <c r="J49" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>2026-05</t>
         </is>
@@ -2767,14 +2832,14 @@
       <c r="I50" s="8" t="n">
         <v>1836</v>
       </c>
-      <c r="J50" s="6" t="inlineStr">
+      <c r="J50" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
@@ -2803,14 +2868,14 @@
       <c r="I51" s="8" t="n">
         <v>2097</v>
       </c>
-      <c r="J51" s="6" t="inlineStr">
+      <c r="J51" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
@@ -2839,14 +2904,14 @@
       <c r="I52" s="8" t="n">
         <v>2202</v>
       </c>
-      <c r="J52" s="6" t="inlineStr">
+      <c r="J52" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
@@ -2875,14 +2940,14 @@
       <c r="I53" s="8" t="n">
         <v>2142</v>
       </c>
-      <c r="J53" s="6" t="inlineStr">
+      <c r="J53" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
@@ -2911,14 +2976,14 @@
       <c r="I54" s="8" t="n">
         <v>2018</v>
       </c>
-      <c r="J54" s="6" t="inlineStr">
+      <c r="J54" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
@@ -2947,14 +3012,14 @@
       <c r="I55" s="8" t="n">
         <v>1914</v>
       </c>
-      <c r="J55" s="6" t="inlineStr">
+      <c r="J55" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>2026-11</t>
         </is>
@@ -2983,7 +3048,7 @@
       <c r="I56" s="8" t="n">
         <v>1938</v>
       </c>
-      <c r="J56" s="6" t="inlineStr">
+      <c r="J56" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
@@ -3022,6 +3087,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Asal: Jakarta (CGK dan HLP); jarak dihitung dari CGK. Semua rute sekali jalan Jakarta → tujuan.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3030,44 +3102,44 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>BPN
-Balikpapan</t>
+          <t>Jakarta →
+BPN Balikpapan</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>DPS
-Denpasar</t>
+          <t>Jakarta →
+DPS Denpasar</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>KNO
-Medan</t>
+          <t>Jakarta →
+KNO Medan</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>PKU
-Pekanbaru</t>
+          <t>Jakarta →
+PKU Pekanbaru</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>SUB
-Surabaya</t>
+          <t>Jakarta →
+SUB Surabaya</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>UPG
-Makassar</t>
+          <t>Jakarta →
+UPG Makassar</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>YIA
-Yogyakarta</t>
+          <t>Jakarta →
+YIA Yogyakarta</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -3082,7 +3154,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>2022-08</t>
         </is>
@@ -3115,14 +3187,14 @@
       <c r="I5" s="8" t="n">
         <v>23</v>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>2022-09</t>
         </is>
@@ -3155,14 +3227,14 @@
       <c r="I6" s="8" t="n">
         <v>71</v>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>2022-10</t>
         </is>
@@ -3195,14 +3267,14 @@
       <c r="I7" s="8" t="n">
         <v>77</v>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>2022-11</t>
         </is>
@@ -3235,14 +3307,14 @@
       <c r="I8" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>2022-12</t>
         </is>
@@ -3275,14 +3347,14 @@
       <c r="I9" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>2023-01</t>
         </is>
@@ -3315,14 +3387,14 @@
       <c r="I10" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>2023-02</t>
         </is>
@@ -3355,14 +3427,14 @@
       <c r="I11" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>2023-03</t>
         </is>
@@ -3395,14 +3467,14 @@
       <c r="I12" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>2023-04</t>
         </is>
@@ -3435,14 +3507,14 @@
       <c r="I13" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>2023-05</t>
         </is>
@@ -3475,14 +3547,14 @@
       <c r="I14" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>2023-06</t>
         </is>
@@ -3515,14 +3587,14 @@
       <c r="I15" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>2023-07</t>
         </is>
@@ -3555,14 +3627,14 @@
       <c r="I16" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>2023-08</t>
         </is>
@@ -3595,14 +3667,14 @@
       <c r="I17" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>2023-09</t>
         </is>
@@ -3635,14 +3707,14 @@
       <c r="I18" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>2023-10</t>
         </is>
@@ -3673,14 +3745,14 @@
       <c r="I19" s="8" t="n">
         <v>267</v>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>2023-11</t>
         </is>
@@ -3709,14 +3781,14 @@
       <c r="I20" s="8" t="n">
         <v>1161</v>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>2023-12</t>
         </is>
@@ -3745,14 +3817,14 @@
       <c r="I21" s="8" t="n">
         <v>2533</v>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J21" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>2024-01</t>
         </is>
@@ -3781,14 +3853,14 @@
       <c r="I22" s="8" t="n">
         <v>2930</v>
       </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>2024-02</t>
         </is>
@@ -3817,14 +3889,14 @@
       <c r="I23" s="8" t="n">
         <v>3542</v>
       </c>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>2024-03</t>
         </is>
@@ -3853,14 +3925,14 @@
       <c r="I24" s="8" t="n">
         <v>4437</v>
       </c>
-      <c r="J24" s="6" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>2024-04</t>
         </is>
@@ -3889,14 +3961,14 @@
       <c r="I25" s="8" t="n">
         <v>3219</v>
       </c>
-      <c r="J25" s="6" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>2024-05</t>
         </is>
@@ -3925,14 +3997,14 @@
       <c r="I26" s="8" t="n">
         <v>3927</v>
       </c>
-      <c r="J26" s="6" t="inlineStr">
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>2024-06</t>
         </is>
@@ -3961,14 +4033,14 @@
       <c r="I27" s="8" t="n">
         <v>3025</v>
       </c>
-      <c r="J27" s="6" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>2024-07</t>
         </is>
@@ -3997,14 +4069,14 @@
       <c r="I28" s="8" t="n">
         <v>3165</v>
       </c>
-      <c r="J28" s="6" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>2024-08</t>
         </is>
@@ -4033,14 +4105,14 @@
       <c r="I29" s="8" t="n">
         <v>3269</v>
       </c>
-      <c r="J29" s="6" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>2024-09</t>
         </is>
@@ -4069,14 +4141,14 @@
       <c r="I30" s="8" t="n">
         <v>1870</v>
       </c>
-      <c r="J30" s="6" t="inlineStr">
+      <c r="J30" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>2024-10</t>
         </is>
@@ -4105,14 +4177,14 @@
       <c r="I31" s="8" t="n">
         <v>1659</v>
       </c>
-      <c r="J31" s="6" t="inlineStr">
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>2024-11</t>
         </is>
@@ -4141,14 +4213,14 @@
       <c r="I32" s="8" t="n">
         <v>2527</v>
       </c>
-      <c r="J32" s="6" t="inlineStr">
+      <c r="J32" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>2024-12</t>
         </is>
@@ -4177,14 +4249,14 @@
       <c r="I33" s="8" t="n">
         <v>2498</v>
       </c>
-      <c r="J33" s="6" t="inlineStr">
+      <c r="J33" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
@@ -4213,14 +4285,14 @@
       <c r="I34" s="8" t="n">
         <v>2385</v>
       </c>
-      <c r="J34" s="6" t="inlineStr">
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>2025-02</t>
         </is>
@@ -4249,14 +4321,14 @@
       <c r="I35" s="8" t="n">
         <v>911</v>
       </c>
-      <c r="J35" s="6" t="inlineStr">
+      <c r="J35" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>2025-03</t>
         </is>
@@ -4285,14 +4357,14 @@
       <c r="I36" s="8" t="n">
         <v>210</v>
       </c>
-      <c r="J36" s="6" t="inlineStr">
+      <c r="J36" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>2025-04</t>
         </is>
@@ -4321,14 +4393,14 @@
       <c r="I37" s="8" t="n">
         <v>494</v>
       </c>
-      <c r="J37" s="6" t="inlineStr">
+      <c r="J37" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
@@ -4357,14 +4429,14 @@
       <c r="I38" s="8" t="n">
         <v>702</v>
       </c>
-      <c r="J38" s="6" t="inlineStr">
+      <c r="J38" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>2025-06</t>
         </is>
@@ -4393,14 +4465,14 @@
       <c r="I39" s="8" t="n">
         <v>636</v>
       </c>
-      <c r="J39" s="6" t="inlineStr">
+      <c r="J39" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>2025-07</t>
         </is>
@@ -4429,14 +4501,14 @@
       <c r="I40" s="8" t="n">
         <v>661</v>
       </c>
-      <c r="J40" s="6" t="inlineStr">
+      <c r="J40" s="5" t="inlineStr">
         <is>
           <t>Traveloka</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>2025-08</t>
         </is>
@@ -4465,14 +4537,14 @@
       <c r="I41" s="8" t="n">
         <v>796</v>
       </c>
-      <c r="J41" s="6" t="inlineStr">
+      <c r="J41" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
@@ -4501,14 +4573,14 @@
       <c r="I42" s="8" t="n">
         <v>337</v>
       </c>
-      <c r="J42" s="6" t="inlineStr">
+      <c r="J42" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>2025-10</t>
         </is>
@@ -4537,14 +4609,14 @@
       <c r="I43" s="8" t="n">
         <v>138</v>
       </c>
-      <c r="J43" s="6" t="inlineStr">
+      <c r="J43" s="5" t="inlineStr">
         <is>
           <t>campuran</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>2025-11</t>
         </is>
@@ -4573,14 +4645,14 @@
       <c r="I44" s="8" t="n">
         <v>104</v>
       </c>
-      <c r="J44" s="6" t="inlineStr">
+      <c r="J44" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
@@ -4609,14 +4681,14 @@
       <c r="I45" s="8" t="n">
         <v>119</v>
       </c>
-      <c r="J45" s="6" t="inlineStr">
+      <c r="J45" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
@@ -4645,14 +4717,14 @@
       <c r="I46" s="8" t="n">
         <v>140</v>
       </c>
-      <c r="J46" s="6" t="inlineStr">
+      <c r="J46" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
@@ -4681,14 +4753,14 @@
       <c r="I47" s="8" t="n">
         <v>112</v>
       </c>
-      <c r="J47" s="6" t="inlineStr">
+      <c r="J47" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
@@ -4717,14 +4789,14 @@
       <c r="I48" s="8" t="n">
         <v>112</v>
       </c>
-      <c r="J48" s="6" t="inlineStr">
+      <c r="J48" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
@@ -4753,14 +4825,14 @@
       <c r="I49" s="8" t="n">
         <v>112</v>
       </c>
-      <c r="J49" s="6" t="inlineStr">
+      <c r="J49" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>2026-05</t>
         </is>
@@ -4789,14 +4861,14 @@
       <c r="I50" s="8" t="n">
         <v>961</v>
       </c>
-      <c r="J50" s="6" t="inlineStr">
+      <c r="J50" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
@@ -4825,14 +4897,14 @@
       <c r="I51" s="8" t="n">
         <v>3610</v>
       </c>
-      <c r="J51" s="6" t="inlineStr">
+      <c r="J51" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
@@ -4861,14 +4933,14 @@
       <c r="I52" s="8" t="n">
         <v>8520</v>
       </c>
-      <c r="J52" s="6" t="inlineStr">
+      <c r="J52" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
@@ -4897,14 +4969,14 @@
       <c r="I53" s="8" t="n">
         <v>8966</v>
       </c>
-      <c r="J53" s="6" t="inlineStr">
+      <c r="J53" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
@@ -4933,14 +5005,14 @@
       <c r="I54" s="8" t="n">
         <v>8099</v>
       </c>
-      <c r="J54" s="6" t="inlineStr">
+      <c r="J54" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
@@ -4969,14 +5041,14 @@
       <c r="I55" s="8" t="n">
         <v>7858</v>
       </c>
-      <c r="J55" s="6" t="inlineStr">
+      <c r="J55" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>2026-11</t>
         </is>
@@ -5005,7 +5077,7 @@
       <c r="I56" s="8" t="n">
         <v>1498</v>
       </c>
-      <c r="J56" s="6" t="inlineStr">
+      <c r="J56" s="5" t="inlineStr">
         <is>
           <t>tiket.com</t>
         </is>
@@ -5022,7 +5094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5036,97 +5108,109 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Rumus</t>
+          <t>Asal &amp; arah</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rp/km = harga tiket ÷ jarak lurus (great-circle) Jakarta (CGK) → bandara tujuan, dirata-rata per kelompok.</t>
+          <t>Semua rute sekali jalan dari Jakarta ke kota tujuan (tidak ada arah sebaliknya). Data Traveloka seluruhnya berangkat dari CGK; data tiket.com mencakup semua bandara Jakarta (sekitar 87% CGK, 13% HLP/Halim). Jarak selalu dihitung dari CGK; selisihnya ke HLP kurang dari 2% sehingga tidak mengubah peringkat.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>Cakupan</t>
+          <t>Rumus</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Hanya penerbangan DIRECT. Penerbangan transit dikeluarkan karena menempuh jarak jauh lebih panjang dari jarak lurus, sehingga Rp/km-nya menyesatkan.</t>
+          <t>Rp/km = harga tiket ÷ jarak lurus (great-circle) Jakarta (CGK) → bandara tujuan, dirata-rata per kelompok.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
+          <t>Cakupan</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Hanya penerbangan DIRECT. Penerbangan transit dikeluarkan karena menempuh jarak jauh lebih panjang dari jarak lurus, sehingga Rp/km-nya menyesatkan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
           <t>Jarak (km)</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>BPN 1.258; DPS 983; KNO 1.387; PKU 933; SUB 691; UPG 1.432; YIA 424; SIN 884; KUL 1.129. Jarak lurus, bukan jarak rute terbang.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Mengapa rute pendek mahal per km</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Biaya tetap per penerbangan (pajak bandara, ground handling) tersebar ke jarak yang lebih pendek, sehingga rute seperti Yogyakarta (424 km) selalu tinggi per km walaupun harga totalnya tidak mahal. Bandingkan antar rute dengan hati-hati; perubahan antar waktu pada rute yang sama lebih bermakna.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
+          <t>Mengapa rute pendek mahal per km</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Biaya tetap per penerbangan (pajak bandara, ground handling) tersebar ke jarak yang lebih pendek, sehingga rute seperti Yogyakarta (424 km) selalu tinggi per km walaupun harga totalnya tidak mahal. Bandingkan antar rute dengan hati-hati; perubahan antar waktu pada rute yang sama lebih bermakna.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
           <t>Sumber &amp; periode</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Arsip Traveloka (Agu 2022 – 2025) dan tiket.com (2026). Dua sumber memiliki cakupan dan komposisi harga berbeda, sehingga ada patahan seri di sekitar Mei 2026 — lihat kolom 'Sumber'. Jangan membaca selisih Apr→Mei 2026 sebagai kenaikan harga murni.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Kenaikan 2026</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Lonjakan Rp/km sejak Mei 2026 bertepatan dengan dua hal: pergantian sumber data dan kenaikan harga avtur akibat guncangan April 2026. Dengan data yang ada keduanya tidak bisa dipisahkan sepenuhnya.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Sampel tipis</t>
+          <t>Kenaikan 2026</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Angka dengan jumlah observasi &lt; 30 ditulis abu-abu miring. Periode Okt 2025 – Apr 2026 memang bersampel tipis (≈110–140 penerbangan per bulan).</t>
+          <t>Lonjakan Rp/km sejak Mei 2026 bertepatan dengan dua hal: pergantian sumber data dan kenaikan harga avtur akibat guncangan April 2026. Dengan data yang ada keduanya tidak bisa dipisahkan sepenuhnya.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
+          <t>Sampel tipis</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Angka dengan jumlah observasi &lt; 30 ditulis abu-abu miring. Periode Okt 2025 – Apr 2026 memang bersampel tipis (≈110–140 penerbangan per bulan).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
           <t>Harga</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Harga tampil untuk 1 penumpang ekonomi sekali jalan; bukan harga tiket yang benar-benar terjual. Penerbangan yang sama dapat terambil di beberapa minggu; semua observasi dirata-rata.</t>
         </is>

</xml_diff>

<commit_message>
Tabulasi Rp/km: tampilkan asal dengan kode CGK
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hasil_scraping/261009-Rp per km per Rute.xlsx
+++ b/hasil_scraping/261009-Rp per km per Rute.xlsx
@@ -531,7 +531,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Asal: Jakarta (CGK dan HLP); jarak dihitung dari CGK. Semua rute sekali jalan Jakarta → tujuan.</t>
+          <t>Asal: Jakarta, kode CGK (sebagian data tiket.com berangkat dari HLP/Halim, ±13%); jarak dihitung dari CGK. Semua rute sekali jalan Jakarta → tujuan.</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>CGK Jakarta</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>CGK Jakarta</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>CGK Jakarta</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>CGK Jakarta</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>CGK Jakarta</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>CGK Jakarta</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>CGK Jakarta</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>CGK Jakarta</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>CGK Jakarta</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1061,7 +1061,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Asal: Jakarta (CGK dan HLP); jarak dihitung dari CGK. Semua rute sekali jalan Jakarta → tujuan.</t>
+          <t>Asal: Jakarta, kode CGK (sebagian data tiket.com berangkat dari HLP/Halim, ±13%); jarak dihitung dari CGK. Semua rute sekali jalan Jakarta → tujuan.</t>
         </is>
       </c>
     </row>
@@ -1073,43 +1073,43 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 BPN Balikpapan</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 DPS Denpasar</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 KNO Medan</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 PKU Pekanbaru</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 SUB Surabaya</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 UPG Makassar</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 YIA Yogyakarta</t>
         </is>
       </c>
@@ -3090,7 +3090,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Asal: Jakarta (CGK dan HLP); jarak dihitung dari CGK. Semua rute sekali jalan Jakarta → tujuan.</t>
+          <t>Asal: Jakarta, kode CGK (sebagian data tiket.com berangkat dari HLP/Halim, ±13%); jarak dihitung dari CGK. Semua rute sekali jalan Jakarta → tujuan.</t>
         </is>
       </c>
     </row>
@@ -3102,43 +3102,43 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 BPN Balikpapan</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 DPS Denpasar</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 KNO Medan</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 PKU Pekanbaru</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 SUB Surabaya</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 UPG Makassar</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Jakarta →
+          <t>CGK →
 YIA Yogyakarta</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Tabulasi Rp/km: potong s.d. Sep 2026, sampel tipis tidak lagi abu-abu
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hasil_scraping/261009-Rp per km per Rute.xlsx
+++ b/hasil_scraping/261009-Rp per km per Rute.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,12 +40,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="0098A2B3"/>
       <sz val="10"/>
     </font>
     <font>
@@ -97,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -112,7 +106,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -478,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1252,13 +1245,13 @@
           <t>2023-10</t>
         </is>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="7" t="n">
         <v>1074</v>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="7" t="n">
         <v>1297</v>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="7" t="n">
         <v>951</v>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -1266,19 +1259,19 @@
           <t>–</t>
         </is>
       </c>
-      <c r="F19" s="10" t="n">
+      <c r="F19" s="7" t="n">
         <v>1674</v>
       </c>
-      <c r="G19" s="10" t="n">
+      <c r="G19" s="7" t="n">
         <v>1157</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>2482</v>
       </c>
-      <c r="I19" s="10" t="n">
+      <c r="I19" s="7" t="n">
         <v>3548</v>
       </c>
-      <c r="J19" s="10" t="n">
+      <c r="J19" s="7" t="n">
         <v>1279</v>
       </c>
       <c r="K19" s="9" t="n">
@@ -1294,31 +1287,31 @@
           <t>2023-11</t>
         </is>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="7" t="n">
         <v>1189</v>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="7" t="n">
         <v>1401</v>
       </c>
-      <c r="D20" s="10" t="n">
+      <c r="D20" s="7" t="n">
         <v>1044</v>
       </c>
-      <c r="E20" s="10" t="n">
+      <c r="E20" s="7" t="n">
         <v>1361</v>
       </c>
-      <c r="F20" s="10" t="n">
+      <c r="F20" s="7" t="n">
         <v>1835</v>
       </c>
-      <c r="G20" s="10" t="n">
+      <c r="G20" s="7" t="n">
         <v>1306</v>
       </c>
-      <c r="H20" s="10" t="n">
+      <c r="H20" s="7" t="n">
         <v>2501</v>
       </c>
-      <c r="I20" s="10" t="n">
+      <c r="I20" s="7" t="n">
         <v>3844</v>
       </c>
-      <c r="J20" s="10" t="n">
+      <c r="J20" s="7" t="n">
         <v>1519</v>
       </c>
       <c r="K20" s="9" t="n">
@@ -1334,31 +1327,31 @@
           <t>2023-12</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="7" t="n">
         <v>1327</v>
       </c>
-      <c r="C21" s="10" t="n">
+      <c r="C21" s="7" t="n">
         <v>1514</v>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="7" t="n">
         <v>1220</v>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="7" t="n">
         <v>1558</v>
       </c>
-      <c r="F21" s="10" t="n">
+      <c r="F21" s="7" t="n">
         <v>1901</v>
       </c>
-      <c r="G21" s="10" t="n">
+      <c r="G21" s="7" t="n">
         <v>1427</v>
       </c>
-      <c r="H21" s="10" t="n">
+      <c r="H21" s="7" t="n">
         <v>2556</v>
       </c>
-      <c r="I21" s="10" t="n">
+      <c r="I21" s="7" t="n">
         <v>4129</v>
       </c>
-      <c r="J21" s="10" t="n">
+      <c r="J21" s="7" t="n">
         <v>1825</v>
       </c>
       <c r="K21" s="9" t="n">
@@ -1374,31 +1367,31 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="B22" s="10" t="n">
+      <c r="B22" s="7" t="n">
         <v>1262</v>
       </c>
-      <c r="C22" s="10" t="n">
+      <c r="C22" s="7" t="n">
         <v>1222</v>
       </c>
-      <c r="D22" s="10" t="n">
+      <c r="D22" s="7" t="n">
         <v>1114</v>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="7" t="n">
         <v>1560</v>
       </c>
-      <c r="F22" s="10" t="n">
+      <c r="F22" s="7" t="n">
         <v>1811</v>
       </c>
-      <c r="G22" s="10" t="n">
+      <c r="G22" s="7" t="n">
         <v>1355</v>
       </c>
-      <c r="H22" s="10" t="n">
+      <c r="H22" s="7" t="n">
         <v>2473</v>
       </c>
-      <c r="I22" s="10" t="n">
+      <c r="I22" s="7" t="n">
         <v>3185</v>
       </c>
-      <c r="J22" s="10" t="n">
+      <c r="J22" s="7" t="n">
         <v>1506</v>
       </c>
       <c r="K22" s="9" t="n">
@@ -1414,31 +1407,31 @@
           <t>2024-02</t>
         </is>
       </c>
-      <c r="B23" s="10" t="n">
+      <c r="B23" s="7" t="n">
         <v>1220</v>
       </c>
-      <c r="C23" s="10" t="n">
+      <c r="C23" s="7" t="n">
         <v>1280</v>
       </c>
-      <c r="D23" s="10" t="n">
+      <c r="D23" s="7" t="n">
         <v>1130</v>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="E23" s="7" t="n">
         <v>1516</v>
       </c>
-      <c r="F23" s="10" t="n">
+      <c r="F23" s="7" t="n">
         <v>1810</v>
       </c>
-      <c r="G23" s="10" t="n">
+      <c r="G23" s="7" t="n">
         <v>1311</v>
       </c>
-      <c r="H23" s="10" t="n">
+      <c r="H23" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="I23" s="10" t="n">
+      <c r="I23" s="7" t="n">
         <v>2748</v>
       </c>
-      <c r="J23" s="10" t="n">
+      <c r="J23" s="7" t="n">
         <v>1573</v>
       </c>
       <c r="K23" s="9" t="n">
@@ -1454,31 +1447,31 @@
           <t>2024-03</t>
         </is>
       </c>
-      <c r="B24" s="10" t="n">
+      <c r="B24" s="7" t="n">
         <v>1242</v>
       </c>
-      <c r="C24" s="10" t="n">
+      <c r="C24" s="7" t="n">
         <v>1217</v>
       </c>
-      <c r="D24" s="10" t="n">
+      <c r="D24" s="7" t="n">
         <v>1197</v>
       </c>
-      <c r="E24" s="10" t="n">
+      <c r="E24" s="7" t="n">
         <v>1525</v>
       </c>
-      <c r="F24" s="10" t="n">
+      <c r="F24" s="7" t="n">
         <v>1771</v>
       </c>
-      <c r="G24" s="10" t="n">
+      <c r="G24" s="7" t="n">
         <v>1342</v>
       </c>
-      <c r="H24" s="10" t="n">
+      <c r="H24" s="7" t="n">
         <v>2402</v>
       </c>
-      <c r="I24" s="10" t="n">
+      <c r="I24" s="7" t="n">
         <v>3110</v>
       </c>
-      <c r="J24" s="10" t="n">
+      <c r="J24" s="7" t="n">
         <v>1432</v>
       </c>
       <c r="K24" s="9" t="n">
@@ -1494,31 +1487,31 @@
           <t>2024-04</t>
         </is>
       </c>
-      <c r="B25" s="10" t="n">
+      <c r="B25" s="7" t="n">
         <v>1379</v>
       </c>
-      <c r="C25" s="10" t="n">
+      <c r="C25" s="7" t="n">
         <v>1439</v>
       </c>
-      <c r="D25" s="10" t="n">
+      <c r="D25" s="7" t="n">
         <v>1216</v>
       </c>
-      <c r="E25" s="10" t="n">
+      <c r="E25" s="7" t="n">
         <v>1587</v>
       </c>
-      <c r="F25" s="10" t="n">
+      <c r="F25" s="7" t="n">
         <v>1899</v>
       </c>
-      <c r="G25" s="10" t="n">
+      <c r="G25" s="7" t="n">
         <v>1435</v>
       </c>
-      <c r="H25" s="10" t="n">
+      <c r="H25" s="7" t="n">
         <v>2507</v>
       </c>
-      <c r="I25" s="10" t="n">
+      <c r="I25" s="7" t="n">
         <v>3876</v>
       </c>
-      <c r="J25" s="10" t="n">
+      <c r="J25" s="7" t="n">
         <v>1845</v>
       </c>
       <c r="K25" s="9" t="n">
@@ -1534,31 +1527,31 @@
           <t>2024-05</t>
         </is>
       </c>
-      <c r="B26" s="10" t="n">
+      <c r="B26" s="7" t="n">
         <v>1366</v>
       </c>
-      <c r="C26" s="10" t="n">
+      <c r="C26" s="7" t="n">
         <v>1353</v>
       </c>
-      <c r="D26" s="10" t="n">
+      <c r="D26" s="7" t="n">
         <v>1132</v>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="E26" s="7" t="n">
         <v>1380</v>
       </c>
-      <c r="F26" s="10" t="n">
+      <c r="F26" s="7" t="n">
         <v>1822</v>
       </c>
-      <c r="G26" s="10" t="n">
+      <c r="G26" s="7" t="n">
         <v>1370</v>
       </c>
-      <c r="H26" s="10" t="n">
+      <c r="H26" s="7" t="n">
         <v>2466</v>
       </c>
-      <c r="I26" s="10" t="n">
+      <c r="I26" s="7" t="n">
         <v>2753</v>
       </c>
-      <c r="J26" s="10" t="n">
+      <c r="J26" s="7" t="n">
         <v>1424</v>
       </c>
       <c r="K26" s="9" t="n">
@@ -1574,31 +1567,31 @@
           <t>2024-06</t>
         </is>
       </c>
-      <c r="B27" s="10" t="n">
+      <c r="B27" s="7" t="n">
         <v>1434</v>
       </c>
-      <c r="C27" s="10" t="n">
+      <c r="C27" s="7" t="n">
         <v>1474</v>
       </c>
-      <c r="D27" s="10" t="n">
+      <c r="D27" s="7" t="n">
         <v>1293</v>
       </c>
-      <c r="E27" s="10" t="n">
+      <c r="E27" s="7" t="n">
         <v>1462</v>
       </c>
-      <c r="F27" s="10" t="n">
+      <c r="F27" s="7" t="n">
         <v>1899</v>
       </c>
-      <c r="G27" s="10" t="n">
+      <c r="G27" s="7" t="n">
         <v>1415</v>
       </c>
-      <c r="H27" s="10" t="n">
+      <c r="H27" s="7" t="n">
         <v>2808</v>
       </c>
-      <c r="I27" s="10" t="n">
+      <c r="I27" s="7" t="n">
         <v>3879</v>
       </c>
-      <c r="J27" s="10" t="n">
+      <c r="J27" s="7" t="n">
         <v>1583</v>
       </c>
       <c r="K27" s="9" t="n">
@@ -1614,31 +1607,31 @@
           <t>2024-07</t>
         </is>
       </c>
-      <c r="B28" s="10" t="n">
+      <c r="B28" s="7" t="n">
         <v>1354</v>
       </c>
-      <c r="C28" s="10" t="n">
+      <c r="C28" s="7" t="n">
         <v>1495</v>
       </c>
-      <c r="D28" s="10" t="n">
+      <c r="D28" s="7" t="n">
         <v>1273</v>
       </c>
-      <c r="E28" s="10" t="n">
+      <c r="E28" s="7" t="n">
         <v>1410</v>
       </c>
-      <c r="F28" s="10" t="n">
+      <c r="F28" s="7" t="n">
         <v>1874</v>
       </c>
-      <c r="G28" s="10" t="n">
+      <c r="G28" s="7" t="n">
         <v>1360</v>
       </c>
-      <c r="H28" s="10" t="n">
+      <c r="H28" s="7" t="n">
         <v>2576</v>
       </c>
-      <c r="I28" s="10" t="n">
+      <c r="I28" s="7" t="n">
         <v>3280</v>
       </c>
-      <c r="J28" s="10" t="n">
+      <c r="J28" s="7" t="n">
         <v>1420</v>
       </c>
       <c r="K28" s="9" t="n">
@@ -1654,31 +1647,31 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="B29" s="10" t="n">
+      <c r="B29" s="7" t="n">
         <v>1328</v>
       </c>
-      <c r="C29" s="10" t="n">
+      <c r="C29" s="7" t="n">
         <v>1501</v>
       </c>
-      <c r="D29" s="10" t="n">
+      <c r="D29" s="7" t="n">
         <v>1247</v>
       </c>
-      <c r="E29" s="10" t="n">
+      <c r="E29" s="7" t="n">
         <v>1326</v>
       </c>
-      <c r="F29" s="10" t="n">
+      <c r="F29" s="7" t="n">
         <v>1959</v>
       </c>
-      <c r="G29" s="10" t="n">
+      <c r="G29" s="7" t="n">
         <v>1355</v>
       </c>
-      <c r="H29" s="10" t="n">
+      <c r="H29" s="7" t="n">
         <v>2753</v>
       </c>
-      <c r="I29" s="10" t="n">
+      <c r="I29" s="7" t="n">
         <v>2951</v>
       </c>
-      <c r="J29" s="10" t="n">
+      <c r="J29" s="7" t="n">
         <v>1382</v>
       </c>
       <c r="K29" s="9" t="n">
@@ -1694,31 +1687,31 @@
           <t>2024-09</t>
         </is>
       </c>
-      <c r="B30" s="10" t="n">
+      <c r="B30" s="7" t="n">
         <v>1247</v>
       </c>
-      <c r="C30" s="10" t="n">
+      <c r="C30" s="7" t="n">
         <v>1525</v>
       </c>
-      <c r="D30" s="10" t="n">
+      <c r="D30" s="7" t="n">
         <v>1277</v>
       </c>
-      <c r="E30" s="10" t="n">
+      <c r="E30" s="7" t="n">
         <v>1370</v>
       </c>
-      <c r="F30" s="10" t="n">
+      <c r="F30" s="7" t="n">
         <v>2173</v>
       </c>
-      <c r="G30" s="10" t="n">
+      <c r="G30" s="7" t="n">
         <v>1419</v>
       </c>
-      <c r="H30" s="10" t="n">
+      <c r="H30" s="7" t="n">
         <v>3104</v>
       </c>
-      <c r="I30" s="10" t="n">
+      <c r="I30" s="7" t="n">
         <v>3712</v>
       </c>
-      <c r="J30" s="10" t="n">
+      <c r="J30" s="7" t="n">
         <v>1510</v>
       </c>
       <c r="K30" s="9" t="n">
@@ -1734,31 +1727,31 @@
           <t>2024-10</t>
         </is>
       </c>
-      <c r="B31" s="10" t="n">
+      <c r="B31" s="7" t="n">
         <v>1166</v>
       </c>
-      <c r="C31" s="10" t="n">
+      <c r="C31" s="7" t="n">
         <v>1439</v>
       </c>
-      <c r="D31" s="10" t="n">
+      <c r="D31" s="7" t="n">
         <v>1220</v>
       </c>
-      <c r="E31" s="10" t="n">
+      <c r="E31" s="7" t="n">
         <v>1318</v>
       </c>
-      <c r="F31" s="10" t="n">
+      <c r="F31" s="7" t="n">
         <v>1960</v>
       </c>
-      <c r="G31" s="10" t="n">
+      <c r="G31" s="7" t="n">
         <v>1395</v>
       </c>
-      <c r="H31" s="10" t="n">
+      <c r="H31" s="7" t="n">
         <v>2861</v>
       </c>
-      <c r="I31" s="10" t="n">
+      <c r="I31" s="7" t="n">
         <v>3096</v>
       </c>
-      <c r="J31" s="10" t="n">
+      <c r="J31" s="7" t="n">
         <v>1170</v>
       </c>
       <c r="K31" s="9" t="n">
@@ -1774,31 +1767,31 @@
           <t>2024-11</t>
         </is>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="7" t="n">
         <v>1205</v>
       </c>
-      <c r="C32" s="10" t="n">
+      <c r="C32" s="7" t="n">
         <v>1465</v>
       </c>
-      <c r="D32" s="10" t="n">
+      <c r="D32" s="7" t="n">
         <v>1232</v>
       </c>
-      <c r="E32" s="10" t="n">
+      <c r="E32" s="7" t="n">
         <v>1344</v>
       </c>
-      <c r="F32" s="10" t="n">
+      <c r="F32" s="7" t="n">
         <v>1997</v>
       </c>
-      <c r="G32" s="10" t="n">
+      <c r="G32" s="7" t="n">
         <v>1408</v>
       </c>
-      <c r="H32" s="10" t="n">
+      <c r="H32" s="7" t="n">
         <v>2803</v>
       </c>
-      <c r="I32" s="10" t="n">
+      <c r="I32" s="7" t="n">
         <v>2659</v>
       </c>
-      <c r="J32" s="10" t="n">
+      <c r="J32" s="7" t="n">
         <v>1143</v>
       </c>
       <c r="K32" s="9" t="n">
@@ -1814,31 +1807,31 @@
           <t>2024-12</t>
         </is>
       </c>
-      <c r="B33" s="10" t="n">
+      <c r="B33" s="7" t="n">
         <v>1221</v>
       </c>
-      <c r="C33" s="10" t="n">
+      <c r="C33" s="7" t="n">
         <v>1455</v>
       </c>
-      <c r="D33" s="10" t="n">
+      <c r="D33" s="7" t="n">
         <v>1319</v>
       </c>
-      <c r="E33" s="10" t="n">
+      <c r="E33" s="7" t="n">
         <v>1478</v>
       </c>
-      <c r="F33" s="10" t="n">
+      <c r="F33" s="7" t="n">
         <v>1956</v>
       </c>
-      <c r="G33" s="10" t="n">
+      <c r="G33" s="7" t="n">
         <v>1689</v>
       </c>
-      <c r="H33" s="10" t="n">
+      <c r="H33" s="7" t="n">
         <v>3018</v>
       </c>
-      <c r="I33" s="10" t="n">
+      <c r="I33" s="7" t="n">
         <v>3812</v>
       </c>
-      <c r="J33" s="10" t="n">
+      <c r="J33" s="7" t="n">
         <v>1610</v>
       </c>
       <c r="K33" s="9" t="n">
@@ -1854,31 +1847,31 @@
           <t>2025-01</t>
         </is>
       </c>
-      <c r="B34" s="10" t="n">
+      <c r="B34" s="7" t="n">
         <v>1260</v>
       </c>
-      <c r="C34" s="10" t="n">
+      <c r="C34" s="7" t="n">
         <v>1293</v>
       </c>
-      <c r="D34" s="10" t="n">
+      <c r="D34" s="7" t="n">
         <v>1167</v>
       </c>
-      <c r="E34" s="10" t="n">
+      <c r="E34" s="7" t="n">
         <v>1443</v>
       </c>
-      <c r="F34" s="10" t="n">
+      <c r="F34" s="7" t="n">
         <v>1994</v>
       </c>
-      <c r="G34" s="10" t="n">
+      <c r="G34" s="7" t="n">
         <v>1869</v>
       </c>
-      <c r="H34" s="10" t="n">
+      <c r="H34" s="7" t="n">
         <v>2947</v>
       </c>
-      <c r="I34" s="10" t="n">
+      <c r="I34" s="7" t="n">
         <v>2470</v>
       </c>
-      <c r="J34" s="10" t="n">
+      <c r="J34" s="7" t="n">
         <v>1272</v>
       </c>
       <c r="K34" s="9" t="n">
@@ -1894,31 +1887,31 @@
           <t>2025-02</t>
         </is>
       </c>
-      <c r="B35" s="10" t="n">
+      <c r="B35" s="7" t="n">
         <v>1302</v>
       </c>
-      <c r="C35" s="10" t="n">
+      <c r="C35" s="7" t="n">
         <v>1381</v>
       </c>
-      <c r="D35" s="10" t="n">
+      <c r="D35" s="7" t="n">
         <v>1285</v>
       </c>
-      <c r="E35" s="10" t="n">
+      <c r="E35" s="7" t="n">
         <v>1426</v>
       </c>
-      <c r="F35" s="10" t="n">
+      <c r="F35" s="7" t="n">
         <v>2216</v>
       </c>
-      <c r="G35" s="10" t="n">
+      <c r="G35" s="7" t="n">
         <v>2115</v>
       </c>
-      <c r="H35" s="10" t="n">
+      <c r="H35" s="7" t="n">
         <v>3266</v>
       </c>
-      <c r="I35" s="10" t="n">
+      <c r="I35" s="7" t="n">
         <v>2139</v>
       </c>
-      <c r="J35" s="10" t="n">
+      <c r="J35" s="7" t="n">
         <v>1292</v>
       </c>
       <c r="K35" s="9" t="n">
@@ -1937,28 +1930,28 @@
       <c r="B36" s="7" t="n">
         <v>1200</v>
       </c>
-      <c r="C36" s="10" t="n">
+      <c r="C36" s="7" t="n">
         <v>1400</v>
       </c>
-      <c r="D36" s="10" t="n">
+      <c r="D36" s="7" t="n">
         <v>1329</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>1440</v>
       </c>
-      <c r="F36" s="10" t="n">
+      <c r="F36" s="7" t="n">
         <v>1977</v>
       </c>
-      <c r="G36" s="10" t="n">
+      <c r="G36" s="7" t="n">
         <v>2368</v>
       </c>
       <c r="H36" s="7" t="n">
         <v>2823</v>
       </c>
-      <c r="I36" s="10" t="n">
+      <c r="I36" s="7" t="n">
         <v>1906</v>
       </c>
-      <c r="J36" s="10" t="n">
+      <c r="J36" s="7" t="n">
         <v>1126</v>
       </c>
       <c r="K36" s="9" t="n">
@@ -1974,31 +1967,31 @@
           <t>2025-04</t>
         </is>
       </c>
-      <c r="B37" s="10" t="n">
+      <c r="B37" s="7" t="n">
         <v>1664</v>
       </c>
-      <c r="C37" s="10" t="n">
+      <c r="C37" s="7" t="n">
         <v>1832</v>
       </c>
-      <c r="D37" s="10" t="n">
+      <c r="D37" s="7" t="n">
         <v>1160</v>
       </c>
-      <c r="E37" s="10" t="n">
+      <c r="E37" s="7" t="n">
         <v>1421</v>
       </c>
-      <c r="F37" s="10" t="n">
+      <c r="F37" s="7" t="n">
         <v>2153</v>
       </c>
-      <c r="G37" s="10" t="n">
+      <c r="G37" s="7" t="n">
         <v>1372</v>
       </c>
-      <c r="H37" s="10" t="n">
+      <c r="H37" s="7" t="n">
         <v>2232</v>
       </c>
-      <c r="I37" s="10" t="n">
+      <c r="I37" s="7" t="n">
         <v>2206</v>
       </c>
-      <c r="J37" s="10" t="n">
+      <c r="J37" s="7" t="n">
         <v>1026</v>
       </c>
       <c r="K37" s="9" t="n">
@@ -2014,31 +2007,31 @@
           <t>2025-05</t>
         </is>
       </c>
-      <c r="B38" s="10" t="n">
+      <c r="B38" s="7" t="n">
         <v>997</v>
       </c>
-      <c r="C38" s="10" t="n">
+      <c r="C38" s="7" t="n">
         <v>1053</v>
       </c>
-      <c r="D38" s="10" t="n">
+      <c r="D38" s="7" t="n">
         <v>945</v>
       </c>
-      <c r="E38" s="10" t="n">
+      <c r="E38" s="7" t="n">
         <v>1284</v>
       </c>
-      <c r="F38" s="10" t="n">
+      <c r="F38" s="7" t="n">
         <v>1405</v>
       </c>
-      <c r="G38" s="10" t="n">
+      <c r="G38" s="7" t="n">
         <v>880</v>
       </c>
-      <c r="H38" s="10" t="n">
+      <c r="H38" s="7" t="n">
         <v>2228</v>
       </c>
-      <c r="I38" s="10" t="n">
+      <c r="I38" s="7" t="n">
         <v>1306</v>
       </c>
-      <c r="J38" s="10" t="n">
+      <c r="J38" s="7" t="n">
         <v>976</v>
       </c>
       <c r="K38" s="9" t="n">
@@ -2054,31 +2047,31 @@
           <t>2025-06</t>
         </is>
       </c>
-      <c r="B39" s="10" t="n">
+      <c r="B39" s="7" t="n">
         <v>1069</v>
       </c>
-      <c r="C39" s="10" t="n">
+      <c r="C39" s="7" t="n">
         <v>1301</v>
       </c>
-      <c r="D39" s="10" t="n">
+      <c r="D39" s="7" t="n">
         <v>1078</v>
       </c>
-      <c r="E39" s="10" t="n">
+      <c r="E39" s="7" t="n">
         <v>1407</v>
       </c>
-      <c r="F39" s="10" t="n">
+      <c r="F39" s="7" t="n">
         <v>1540</v>
       </c>
-      <c r="G39" s="10" t="n">
+      <c r="G39" s="7" t="n">
         <v>1032</v>
       </c>
-      <c r="H39" s="10" t="n">
+      <c r="H39" s="7" t="n">
         <v>2468</v>
       </c>
-      <c r="I39" s="10" t="n">
+      <c r="I39" s="7" t="n">
         <v>1457</v>
       </c>
-      <c r="J39" s="10" t="n">
+      <c r="J39" s="7" t="n">
         <v>1092</v>
       </c>
       <c r="K39" s="9" t="n">
@@ -2094,31 +2087,31 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="B40" s="10" t="n">
+      <c r="B40" s="7" t="n">
         <v>1027</v>
       </c>
-      <c r="C40" s="10" t="n">
+      <c r="C40" s="7" t="n">
         <v>1297</v>
       </c>
-      <c r="D40" s="10" t="n">
+      <c r="D40" s="7" t="n">
         <v>1028</v>
       </c>
-      <c r="E40" s="10" t="n">
+      <c r="E40" s="7" t="n">
         <v>1324</v>
       </c>
-      <c r="F40" s="10" t="n">
+      <c r="F40" s="7" t="n">
         <v>1514</v>
       </c>
-      <c r="G40" s="10" t="n">
+      <c r="G40" s="7" t="n">
         <v>1179</v>
       </c>
-      <c r="H40" s="10" t="n">
+      <c r="H40" s="7" t="n">
         <v>2392</v>
       </c>
-      <c r="I40" s="10" t="n">
+      <c r="I40" s="7" t="n">
         <v>1153</v>
       </c>
-      <c r="J40" s="10" t="n">
+      <c r="J40" s="7" t="n">
         <v>1164</v>
       </c>
       <c r="K40" s="9" t="n">
@@ -2134,31 +2127,31 @@
           <t>2025-08</t>
         </is>
       </c>
-      <c r="B41" s="10" t="n">
+      <c r="B41" s="7" t="n">
         <v>985</v>
       </c>
-      <c r="C41" s="10" t="n">
+      <c r="C41" s="7" t="n">
         <v>1326</v>
       </c>
-      <c r="D41" s="10" t="n">
+      <c r="D41" s="7" t="n">
         <v>934</v>
       </c>
-      <c r="E41" s="10" t="n">
+      <c r="E41" s="7" t="n">
         <v>1317</v>
       </c>
-      <c r="F41" s="10" t="n">
+      <c r="F41" s="7" t="n">
         <v>1509</v>
       </c>
-      <c r="G41" s="10" t="n">
+      <c r="G41" s="7" t="n">
         <v>884</v>
       </c>
-      <c r="H41" s="10" t="n">
+      <c r="H41" s="7" t="n">
         <v>2396</v>
       </c>
-      <c r="I41" s="10" t="n">
+      <c r="I41" s="7" t="n">
         <v>1029</v>
       </c>
-      <c r="J41" s="10" t="n">
+      <c r="J41" s="7" t="n">
         <v>929</v>
       </c>
       <c r="K41" s="9" t="n">
@@ -2174,31 +2167,31 @@
           <t>2025-09</t>
         </is>
       </c>
-      <c r="B42" s="10" t="n">
+      <c r="B42" s="7" t="n">
         <v>1019</v>
       </c>
-      <c r="C42" s="10" t="n">
+      <c r="C42" s="7" t="n">
         <v>1276</v>
       </c>
-      <c r="D42" s="10" t="n">
+      <c r="D42" s="7" t="n">
         <v>932</v>
       </c>
-      <c r="E42" s="10" t="n">
+      <c r="E42" s="7" t="n">
         <v>1429</v>
       </c>
-      <c r="F42" s="10" t="n">
+      <c r="F42" s="7" t="n">
         <v>1474</v>
       </c>
-      <c r="G42" s="10" t="n">
+      <c r="G42" s="7" t="n">
         <v>1331</v>
       </c>
-      <c r="H42" s="10" t="n">
+      <c r="H42" s="7" t="n">
         <v>2385</v>
       </c>
-      <c r="I42" s="10" t="n">
+      <c r="I42" s="7" t="n">
         <v>1052</v>
       </c>
-      <c r="J42" s="10" t="n">
+      <c r="J42" s="7" t="n">
         <v>1045</v>
       </c>
       <c r="K42" s="9" t="n">
@@ -2494,31 +2487,31 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="B50" s="10" t="n">
+      <c r="B50" s="7" t="n">
         <v>1479</v>
       </c>
-      <c r="C50" s="10" t="n">
+      <c r="C50" s="7" t="n">
         <v>1977</v>
       </c>
-      <c r="D50" s="10" t="n">
+      <c r="D50" s="7" t="n">
         <v>1356</v>
       </c>
-      <c r="E50" s="10" t="n">
+      <c r="E50" s="7" t="n">
         <v>1744</v>
       </c>
-      <c r="F50" s="10" t="n">
+      <c r="F50" s="7" t="n">
         <v>2201</v>
       </c>
-      <c r="G50" s="10" t="n">
+      <c r="G50" s="7" t="n">
         <v>1438</v>
       </c>
-      <c r="H50" s="10" t="n">
+      <c r="H50" s="7" t="n">
         <v>2881</v>
       </c>
-      <c r="I50" s="10" t="n">
+      <c r="I50" s="7" t="n">
         <v>3091</v>
       </c>
-      <c r="J50" s="10" t="n">
+      <c r="J50" s="7" t="n">
         <v>2015</v>
       </c>
       <c r="K50" s="9" t="n">
@@ -2534,31 +2527,31 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B51" s="10" t="n">
+      <c r="B51" s="7" t="n">
         <v>1689</v>
       </c>
-      <c r="C51" s="10" t="n">
+      <c r="C51" s="7" t="n">
         <v>2130</v>
       </c>
-      <c r="D51" s="10" t="n">
+      <c r="D51" s="7" t="n">
         <v>1683</v>
       </c>
-      <c r="E51" s="10" t="n">
+      <c r="E51" s="7" t="n">
         <v>2043</v>
       </c>
-      <c r="F51" s="10" t="n">
+      <c r="F51" s="7" t="n">
         <v>2482</v>
       </c>
-      <c r="G51" s="10" t="n">
+      <c r="G51" s="7" t="n">
         <v>1703</v>
       </c>
-      <c r="H51" s="10" t="n">
+      <c r="H51" s="7" t="n">
         <v>3223</v>
       </c>
-      <c r="I51" s="10" t="n">
+      <c r="I51" s="7" t="n">
         <v>4029</v>
       </c>
-      <c r="J51" s="10" t="n">
+      <c r="J51" s="7" t="n">
         <v>2469</v>
       </c>
       <c r="K51" s="9" t="n">
@@ -2574,31 +2567,31 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="B52" s="10" t="n">
+      <c r="B52" s="7" t="n">
         <v>1792</v>
       </c>
-      <c r="C52" s="10" t="n">
+      <c r="C52" s="7" t="n">
         <v>2197</v>
       </c>
-      <c r="D52" s="10" t="n">
+      <c r="D52" s="7" t="n">
         <v>1769</v>
       </c>
-      <c r="E52" s="10" t="n">
+      <c r="E52" s="7" t="n">
         <v>2117</v>
       </c>
-      <c r="F52" s="10" t="n">
+      <c r="F52" s="7" t="n">
         <v>2601</v>
       </c>
-      <c r="G52" s="10" t="n">
+      <c r="G52" s="7" t="n">
         <v>1767</v>
       </c>
-      <c r="H52" s="10" t="n">
+      <c r="H52" s="7" t="n">
         <v>3435</v>
       </c>
-      <c r="I52" s="10" t="n">
+      <c r="I52" s="7" t="n">
         <v>3017</v>
       </c>
-      <c r="J52" s="10" t="n">
+      <c r="J52" s="7" t="n">
         <v>1889</v>
       </c>
       <c r="K52" s="9" t="n">
@@ -2614,31 +2607,31 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="B53" s="10" t="n">
+      <c r="B53" s="7" t="n">
         <v>1764</v>
       </c>
-      <c r="C53" s="10" t="n">
+      <c r="C53" s="7" t="n">
         <v>2210</v>
       </c>
-      <c r="D53" s="10" t="n">
+      <c r="D53" s="7" t="n">
         <v>1694</v>
       </c>
-      <c r="E53" s="10" t="n">
+      <c r="E53" s="7" t="n">
         <v>2064</v>
       </c>
-      <c r="F53" s="10" t="n">
+      <c r="F53" s="7" t="n">
         <v>2517</v>
       </c>
-      <c r="G53" s="10" t="n">
+      <c r="G53" s="7" t="n">
         <v>1693</v>
       </c>
-      <c r="H53" s="10" t="n">
+      <c r="H53" s="7" t="n">
         <v>3277</v>
       </c>
-      <c r="I53" s="10" t="n">
+      <c r="I53" s="7" t="n">
         <v>3384</v>
       </c>
-      <c r="J53" s="10" t="n">
+      <c r="J53" s="7" t="n">
         <v>1993</v>
       </c>
       <c r="K53" s="9" t="n">
@@ -2654,31 +2647,31 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="B54" s="10" t="n">
+      <c r="B54" s="7" t="n">
         <v>1710</v>
       </c>
-      <c r="C54" s="10" t="n">
+      <c r="C54" s="7" t="n">
         <v>2032</v>
       </c>
-      <c r="D54" s="10" t="n">
+      <c r="D54" s="7" t="n">
         <v>1553</v>
       </c>
-      <c r="E54" s="10" t="n">
+      <c r="E54" s="7" t="n">
         <v>1949</v>
       </c>
-      <c r="F54" s="10" t="n">
+      <c r="F54" s="7" t="n">
         <v>2405</v>
       </c>
-      <c r="G54" s="10" t="n">
+      <c r="G54" s="7" t="n">
         <v>1601</v>
       </c>
-      <c r="H54" s="10" t="n">
+      <c r="H54" s="7" t="n">
         <v>3080</v>
       </c>
-      <c r="I54" s="10" t="n">
+      <c r="I54" s="7" t="n">
         <v>2542</v>
       </c>
-      <c r="J54" s="10" t="n">
+      <c r="J54" s="7" t="n">
         <v>1892</v>
       </c>
       <c r="K54" s="9" t="n">
@@ -2686,86 +2679,6 @@
       </c>
       <c r="L54" s="9" t="n">
         <v>2213</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B55" s="10" t="n">
-        <v>1601</v>
-      </c>
-      <c r="C55" s="10" t="n">
-        <v>1951</v>
-      </c>
-      <c r="D55" s="10" t="n">
-        <v>1453</v>
-      </c>
-      <c r="E55" s="10" t="n">
-        <v>1778</v>
-      </c>
-      <c r="F55" s="10" t="n">
-        <v>2248</v>
-      </c>
-      <c r="G55" s="10" t="n">
-        <v>1586</v>
-      </c>
-      <c r="H55" s="10" t="n">
-        <v>2911</v>
-      </c>
-      <c r="I55" s="10" t="n">
-        <v>2332</v>
-      </c>
-      <c r="J55" s="10" t="n">
-        <v>1911</v>
-      </c>
-      <c r="K55" s="9" t="n">
-        <v>1914</v>
-      </c>
-      <c r="L55" s="9" t="n">
-        <v>2112</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>2026-11</t>
-        </is>
-      </c>
-      <c r="B56" s="10" t="n">
-        <v>1582</v>
-      </c>
-      <c r="C56" s="10" t="n">
-        <v>1929</v>
-      </c>
-      <c r="D56" s="10" t="n">
-        <v>1424</v>
-      </c>
-      <c r="E56" s="10" t="n">
-        <v>1788</v>
-      </c>
-      <c r="F56" s="10" t="n">
-        <v>2415</v>
-      </c>
-      <c r="G56" s="10" t="n">
-        <v>1618</v>
-      </c>
-      <c r="H56" s="10" t="n">
-        <v>2796</v>
-      </c>
-      <c r="I56" s="10" t="n">
-        <v>2275</v>
-      </c>
-      <c r="J56" s="10" t="n">
-        <v>1758</v>
-      </c>
-      <c r="K56" s="9" t="n">
-        <v>1938</v>
-      </c>
-      <c r="L56" s="9" t="n">
-        <v>1981</v>
       </c>
     </row>
   </sheetData>

</xml_diff>